<commit_message>
docs(cp3): model five cost components and pricing sensitivity
</commit_message>
<xml_diff>
--- a/deliverables/Day22-DevPulse-Monetization-Model.xlsx
+++ b/deliverables/Day22-DevPulse-Monetization-Model.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Assumptions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7_Assumptions'!$A$3:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7_Assumptions'!$A$3:$F$69</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -98,7 +98,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +135,16 @@
         <bgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border/>
@@ -162,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -311,7 +321,25 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -393,6 +421,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>None</author>
+    <author>Day22 provenance</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0">
@@ -403,11 +432,96 @@
 Ví dụ mẫu đang điền sẵn — thay bằng sản phẩm của bạn.</t>
       </text>
     </comment>
+    <comment ref="B9" authorId="1" shapeId="0">
+      <text>
+        <t>Planning: 10 workspaces × 4 attempted reports/month = 40. Day20 cadence: two sprint reports and one board report delivered. Not current customers.</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="1" shapeId="0">
+      <text>
+        <t>75% planning assumption, not eval. 40 attempts → 30 AI-ready. CTO review remains mandatory; preparation containment ≠ end-to-end autonomy.</t>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="1" shapeId="0">
+      <text>
+        <t>8,000 stable prefix tokens ≥ Haiku 4.5 cache minimum 4,096. Four sequential calls within five-minute TTL. No claim measured hit rate.</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="1" shapeId="0">
+      <text>
+        <t>12,000 average fresh tokens/call includes history, structured source aggregates, tool schemas and results; no raw source-code ingestion. Must replace with usage logs.</t>
+      </text>
+    </comment>
+    <comment ref="B30" authorId="1" shapeId="0">
+      <text>
+        <t>No Batch in baseline: planned on-demand preview within 15 minutes. Batch scenario only for overnight reports, no assumed cache sharing across batched jobs.</t>
+      </text>
+    </comment>
+    <comment ref="B41" authorId="1" shapeId="0">
+      <text>
+        <t>$80 shared monthly floor / 40 attempts + $8 per attempt = $10. $8: ingestion/DB $3, storage/egress $1, logging/eval $1, direct support $1.5, collection/FX/tax contingency $1.5. Estimates, not invoices.</t>
+      </text>
+    </comment>
+    <comment ref="B46" authorId="1" shapeId="0">
+      <text>
+        <t>8% assumes exactly one extra full inference per affected job. More repeats require expected extra call count, not probability alone. Infra retry reserve in logging component.</t>
+      </text>
+    </comment>
+    <comment ref="B50" authorId="1" shapeId="0">
+      <text>
+        <t>Fully-loaded vendor QA/support $20/hour is planning assumption, not Vietnam wage benchmark.</t>
+      </text>
+    </comment>
+    <comment ref="B53" authorId="1" shapeId="0">
+      <text>
+        <t>20 minutes/customer-reworked failure is a scenario input. Vendor cost = zero only in variant A; customer burden must be measured.</t>
+      </text>
+    </comment>
+    <comment ref="B59" authorId="1" shapeId="0">
+      <text>
+        <t>$300/month allocation: ongoing product maintenance 8h×$20 + admin 7h×$20. Acquisition spend is in CAC, not double-counted here. Not complete startup payroll.</t>
+      </text>
+    </comment>
+    <comment ref="B68" authorId="1" shapeId="0">
+      <text>
+        <t>Vietcombank XML USD sell 26,160 VND/USD; published 10/8/2026 12:13:07 PM; checked 2026-10-08. Excludes payment fees.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Day22 provenance</author>
+  </authors>
+  <commentList>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>3 reports/month × 10 net preparation hours saved × $40/hour = $1,200. No token-spend savings or causal developer productivity claim. Pilot stopwatch required.</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>AI-ready reports/customer/month, not attempted reports. Three reports follows two sprint reports + one monthly board review from Day20.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Hypothetical reporting analyst $2,000/month; not an employee actually replaced. Primary anchor is saved preparation hours.</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>$60/report, hypothesis: above 3×COGS floor; at 3 reports plus $39 base, $219/month &lt; 25% of $1,200 saved. WTP unvalidated.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Day22 provenance</author>
@@ -2002,7 +2116,7 @@
           <t>Giá input ($ / 1M token)</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="50" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="17" t="inlineStr">
@@ -2017,7 +2131,7 @@
           <t>Giá output ($ / 1M token)</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="50" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2027,7 +2141,7 @@
           <t>Giá cache WRITE ($ / 1M token)</t>
         </is>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B17" s="50" t="n">
         <v>1.25</v>
       </c>
       <c r="D17" s="17" t="inlineStr">
@@ -2042,7 +2156,7 @@
           <t>Giá cache READ ($ / 1M token)</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n">
+      <c r="B18" s="50" t="n">
         <v>0.1</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
@@ -2057,8 +2171,8 @@
           <t>Số lượt (turns) / job</t>
         </is>
       </c>
-      <c r="B19" s="15" t="n">
-        <v>6</v>
+      <c r="B19" s="48" t="n">
+        <v>4</v>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
@@ -2072,8 +2186,8 @@
           <t>Token input CACHE ĐƯỢC / lượt</t>
         </is>
       </c>
-      <c r="B20" s="15" t="n">
-        <v>3000</v>
+      <c r="B20" s="48" t="n">
+        <v>8000</v>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
@@ -2092,8 +2206,8 @@
           <t>Token input FRESH / lượt</t>
         </is>
       </c>
-      <c r="B21" s="15" t="n">
-        <v>1000</v>
+      <c r="B21" s="48" t="n">
+        <v>12000</v>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
@@ -2112,8 +2226,8 @@
           <t>Token output / lượt</t>
         </is>
       </c>
-      <c r="B22" s="15" t="n">
-        <v>300</v>
+      <c r="B22" s="48" t="n">
+        <v>2000</v>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
@@ -2209,7 +2323,7 @@
           <t>Dùng Batch API? (1 = có, 0 = không)</t>
         </is>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B30" s="48" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="17" t="inlineStr">
@@ -2250,7 +2364,7 @@
           <t>Giá STT ($ / phút)</t>
         </is>
       </c>
-      <c r="B34" s="29" t="n">
+      <c r="B34" s="51" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="17" t="inlineStr">
@@ -2265,7 +2379,7 @@
           <t>Số phút audio / job</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n">
+      <c r="B35" s="52" t="n">
         <v>0</v>
       </c>
       <c r="C35" s="17" t="inlineStr">
@@ -2280,7 +2394,7 @@
           <t>Giá TTS ($ / 1M ký tự)</t>
         </is>
       </c>
-      <c r="B36" s="22" t="n">
+      <c r="B36" s="50" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="17" t="inlineStr">
@@ -2295,7 +2409,7 @@
           <t>Số ký tự TTS / job</t>
         </is>
       </c>
-      <c r="B37" s="15" t="n">
+      <c r="B37" s="48" t="n">
         <v>0</v>
       </c>
       <c r="C37" s="17" t="inlineStr">
@@ -2341,8 +2455,8 @@
           <t>Infra / job ($)</t>
         </is>
       </c>
-      <c r="B41" s="29" t="n">
-        <v>0.005</v>
+      <c r="B41" s="51" t="n">
+        <v>10</v>
       </c>
       <c r="D41" s="17" t="inlineStr">
         <is>
@@ -2356,7 +2470,7 @@
           <t>Telephony ($ / phút)</t>
         </is>
       </c>
-      <c r="B42" s="29" t="n">
+      <c r="B42" s="51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2392,7 +2506,7 @@
           <t>Tỷ lệ job phải chạy lại</t>
         </is>
       </c>
-      <c r="B46" s="16" t="n">
+      <c r="B46" s="49" t="n">
         <v>0.08</v>
       </c>
       <c r="D46" s="17" t="inlineStr">
@@ -2433,8 +2547,8 @@
           <t>Chi phí nhân sự ($ / giờ, fully-loaded)</t>
         </is>
       </c>
-      <c r="B50" s="22" t="n">
-        <v>9</v>
+      <c r="B50" s="50" t="n">
+        <v>20</v>
       </c>
       <c r="D50" s="17" t="inlineStr">
         <is>
@@ -2448,8 +2562,8 @@
           <t>% hội thoại QA nội bộ</t>
         </is>
       </c>
-      <c r="B51" s="16" t="n">
-        <v>0.05</v>
+      <c r="B51" s="49" t="n">
+        <v>0.25</v>
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
@@ -2463,8 +2577,8 @@
           <t>Số phút QA / ca</t>
         </is>
       </c>
-      <c r="B52" s="21" t="n">
-        <v>2</v>
+      <c r="B52" s="52" t="n">
+        <v>15</v>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
@@ -2478,8 +2592,8 @@
           <t>Số phút xử lý 1 ca escalate</t>
         </is>
       </c>
-      <c r="B53" s="21" t="n">
-        <v>6</v>
+      <c r="B53" s="52" t="n">
+        <v>20</v>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
@@ -2546,8 +2660,8 @@
           <t>R&amp;D + Sales phân bổ / tháng ($)</t>
         </is>
       </c>
-      <c r="B59" s="22" t="n">
-        <v>0</v>
+      <c r="B59" s="50" t="n">
+        <v>300</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
@@ -2657,8 +2771,8 @@
           <t>Tỷ giá (₫ / USD) — giả định</t>
         </is>
       </c>
-      <c r="B68" s="15" t="n">
-        <v>26000</v>
+      <c r="B68" s="48" t="n">
+        <v>26160</v>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
@@ -3806,7 +3920,7 @@
           <t>Hệ số an toàn tối thiểu</t>
         </is>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="52" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
@@ -3856,8 +3970,8 @@
           <t>Giá trị khách tiết kiệm được / tháng ($)</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n">
-        <v>4000</v>
+      <c r="B10" s="53" t="n">
+        <v>1200</v>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
@@ -3871,8 +3985,8 @@
           <t>Số job / tháng của 1 khách</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
-        <v>1000</v>
+      <c r="B11" s="48" t="n">
+        <v>3</v>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
@@ -3918,8 +4032,8 @@
           <t>Lương / tháng của vị trí bị thay ($)</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n">
-        <v>1500</v>
+      <c r="B14" s="53" t="n">
+        <v>2000</v>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
@@ -3979,8 +4093,8 @@
           <t>★ Giá bán đề xuất ($ / job)</t>
         </is>
       </c>
-      <c r="B19" s="29" t="n">
-        <v>0.99</v>
+      <c r="B19" s="51" t="n">
+        <v>60</v>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
@@ -4120,7 +4234,7 @@
           <t>Gross Margin mục tiêu</t>
         </is>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B32" s="49" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -5329,6 +5443,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -11504,7 +11619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="45" min="1" max="1"/>
@@ -11516,63 +11631,2092 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="50" t="inlineStr">
+      <c r="A1" s="54" t="inlineStr">
         <is>
           <t>DAY22 — DEVPULSE: ASSUMPTIONS &amp; TRACEABILITY</t>
         </is>
       </c>
-      <c r="B1" s="50" t="n"/>
-      <c r="C1" s="50" t="n"/>
-      <c r="D1" s="50" t="n"/>
-      <c r="E1" s="50" t="n"/>
-      <c r="F1" s="50" t="n"/>
+      <c r="B1" s="54" t="n"/>
+      <c r="C1" s="54" t="n"/>
+      <c r="D1" s="54" t="n"/>
+      <c r="E1" s="54" t="n"/>
+      <c r="F1" s="54" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="50" t="inlineStr">
+      <c r="A2" s="54" t="inlineStr">
         <is>
           <t>Giả định vận hành ≠ eval thực đo. Các tab gốc giữ nguyên giá trị ngoài ô vàng.</t>
         </is>
       </c>
-      <c r="B2" s="50" t="n"/>
-      <c r="C2" s="50" t="n"/>
-      <c r="D2" s="50" t="n"/>
-      <c r="E2" s="50" t="n"/>
-      <c r="F2" s="50" t="n"/>
+      <c r="B2" s="54" t="n"/>
+      <c r="C2" s="54" t="n"/>
+      <c r="D2" s="54" t="n"/>
+      <c r="E2" s="54" t="n"/>
+      <c r="F2" s="54" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="54" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B3" s="50" t="inlineStr">
+      <c r="B3" s="54" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C3" s="50" t="inlineStr">
+      <c r="C3" s="54" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D3" s="50" t="inlineStr">
+      <c r="D3" s="54" t="inlineStr">
         <is>
           <t>Evidence status</t>
         </is>
       </c>
-      <c r="E3" s="50" t="inlineStr">
+      <c r="E3" s="54" t="inlineStr">
         <is>
           <t>Rationale / verification</t>
         </is>
       </c>
-      <c r="F3" s="50" t="inlineStr">
+      <c r="F3" s="54" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="48" customHeight="1" s="45">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="inlineStr">
+        <is>
+          <t>DevPulse AI</t>
+        </is>
+      </c>
+      <c r="C4" s="54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D4" s="54" t="inlineStr">
+        <is>
+          <t>Day20 specification</t>
+        </is>
+      </c>
+      <c r="E4" s="54" t="inlineStr">
+        <is>
+          <t>CTO engineering and AI-cost reporting</t>
+        </is>
+      </c>
+      <c r="F4" s="54" t="inlineStr">
+        <is>
+          <t>data/day20-metrics-pack.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1" s="45">
+      <c r="A5" s="54" t="inlineStr">
+        <is>
+          <t>ICP minimum developers</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>developers</t>
+        </is>
+      </c>
+      <c r="D5" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>Narrow growth-team ICP; validate interviews</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t>Day20 segments</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1" s="45">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>ICP maximum developers</t>
+        </is>
+      </c>
+      <c r="B6" s="55" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>developers</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E6" s="54" t="inlineStr">
+        <is>
+          <t>Do not claim validated market</t>
+        </is>
+      </c>
+      <c r="F6" s="54" t="inlineStr">
+        <is>
+          <t>Day20 segments</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" s="45">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
+          <t>Budget owner</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="inlineStr">
+        <is>
+          <t>CTO; CEO/CFO per approval limit</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E7" s="54" t="inlineStr">
+        <is>
+          <t>Pilot confirms actual signer</t>
+        </is>
+      </c>
+      <c r="F7" s="54" t="inlineStr">
+        <is>
+          <t>docs/checkpoints/01-budget-job.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" s="45">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>Budget line</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="inlineStr">
+        <is>
+          <t>Engineering Operations / Reporting</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E8" s="54" t="inlineStr">
+        <is>
+          <t>Time spent consolidating reporting</t>
+        </is>
+      </c>
+      <c r="F8" s="54" t="inlineStr">
+        <is>
+          <t>docs/checkpoints/01-budget-job.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" s="45">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>Positioning</t>
+        </is>
+      </c>
+      <c r="B9" s="55" t="inlineStr">
+        <is>
+          <t>Chuẩn bị báo cáo Sprint/tháng có nguồn để CTO giải trình delivery và chi phí AI.</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="E9" s="54" t="inlineStr">
+        <is>
+          <t>Not causal ROI outcome</t>
+        </is>
+      </c>
+      <c r="F9" s="54" t="inlineStr">
+        <is>
+          <t>Day20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" s="45">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Workspace base fee</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>39</v>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>USD/workspace/month</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>pricing hypothesis</t>
+        </is>
+      </c>
+      <c r="E10" s="54" t="inlineStr">
+        <is>
+          <t>Connections, history, standard support; zero included reports</t>
+        </is>
+      </c>
+      <c r="F10" s="54" t="inlineStr">
+        <is>
+          <t>Decision Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" s="45">
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t>Reports/customer/month</t>
+        </is>
+      </c>
+      <c r="B11" s="56">
+        <f>'2_Pricing'!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>reports</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>planning</t>
+        </is>
+      </c>
+      <c r="E11" s="54" t="inlineStr">
+        <is>
+          <t>2 sprint + 1 board report; average delivered</t>
+        </is>
+      </c>
+      <c r="F11" s="54" t="inlineStr">
+        <is>
+          <t>Day20 cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" s="45">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
+          <t>Planning workspaces</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>workspaces</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
+        <is>
+          <t>Target steady planning cohort, not current users</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr">
+        <is>
+          <t>90-day plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" s="45">
+      <c r="A13" s="54" t="inlineStr">
+        <is>
+          <t>Attempts/workspace/month</t>
+        </is>
+      </c>
+      <c r="B13" s="56">
+        <f>'1_Cost_Job'!B9/B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>attempts</t>
+        </is>
+      </c>
+      <c r="D13" s="54" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E13" s="54" t="inlineStr">
+        <is>
+          <t>40 attempts allocated to 10 workspaces</t>
+        </is>
+      </c>
+      <c r="F13" s="54" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" s="45">
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>Data coverage gate</t>
+        </is>
+      </c>
+      <c r="B14" s="55" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="E14" s="54" t="inlineStr">
+        <is>
+          <t>Coverage of active developers; suppress report if missing ledger</t>
+        </is>
+      </c>
+      <c r="F14" s="54" t="inlineStr">
+        <is>
+          <t>Day20 NSM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" s="45">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>Internal QA sample</t>
+        </is>
+      </c>
+      <c r="B15" s="56">
+        <f>'1_Cost_Job'!B51</f>
+        <v/>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E15" s="54" t="inlineStr">
+        <is>
+          <t>25% sample while early; customer final review every report</t>
+        </is>
+      </c>
+      <c r="F15" s="54" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B51</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" s="45">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
+          <t>Customer review minutes</t>
+        </is>
+      </c>
+      <c r="B16" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>minutes/report</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>Day20 specification</t>
+        </is>
+      </c>
+      <c r="E16" s="54" t="inlineStr">
+        <is>
+          <t>Not replaced by AI; cost borne by customer</t>
+        </is>
+      </c>
+      <c r="F16" s="54" t="inlineStr">
+        <is>
+          <t>Day20 action effort 15–30min</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" s="45">
+      <c r="A17" s="54" t="inlineStr">
+        <is>
+          <t>Net preparation hours saved/report</t>
+        </is>
+      </c>
+      <c r="B17" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E17" s="54" t="inlineStr">
+        <is>
+          <t>Excludes final CTO review; stopwatch before/after</t>
+        </is>
+      </c>
+      <c r="F17" s="54" t="inlineStr">
+        <is>
+          <t>Pilot Protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" s="45">
+      <c r="A18" s="54" t="inlineStr">
+        <is>
+          <t>Customer preparation labor</t>
+        </is>
+      </c>
+      <c r="B18" s="55" t="n">
+        <v>40</v>
+      </c>
+      <c r="C18" s="54" t="inlineStr">
+        <is>
+          <t>USD/hour</t>
+        </is>
+      </c>
+      <c r="D18" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E18" s="54" t="inlineStr">
+        <is>
+          <t>Fully loaded lead/analyst time; no wage benchmark claim</t>
+        </is>
+      </c>
+      <c r="F18" s="54" t="inlineStr">
+        <is>
+          <t>Pilot interview required</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" s="45">
+      <c r="A19" s="54" t="inlineStr">
+        <is>
+          <t>Monthly value anchor</t>
+        </is>
+      </c>
+      <c r="B19" s="56">
+        <f>B11*B17*B18</f>
+        <v/>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D19" s="54" t="inlineStr">
+        <is>
+          <t>derived estimate</t>
+        </is>
+      </c>
+      <c r="E19" s="54" t="inlineStr">
+        <is>
+          <t>No double-counting token or productivity savings</t>
+        </is>
+      </c>
+      <c r="F19" s="54" t="inlineStr">
+        <is>
+          <t>2_Pricing!B10</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" s="45">
+      <c r="A20" s="54" t="inlineStr">
+        <is>
+          <t>Reporting role wage</t>
+        </is>
+      </c>
+      <c r="B20" s="56">
+        <f>'2_Pricing'!B14</f>
+        <v/>
+      </c>
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D20" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E20" s="54" t="inlineStr">
+        <is>
+          <t>Secondary anchor only; no whole role replacement claim</t>
+        </is>
+      </c>
+      <c r="F20" s="54" t="inlineStr">
+        <is>
+          <t>2_Pricing!B14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" s="45">
+      <c r="A21" s="54" t="inlineStr">
+        <is>
+          <t>Monthly vendor COGS</t>
+        </is>
+      </c>
+      <c r="B21" s="56">
+        <f>'1_Cost_Job'!B62+'1_Cost_Job'!B63</f>
+        <v/>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D21" s="54" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E21" s="54" t="inlineStr">
+        <is>
+          <t>All direct service costs</t>
+        </is>
+      </c>
+      <c r="F21" s="54" t="inlineStr">
+        <is>
+          <t>1_Cost_Job</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" s="45">
+      <c r="A22" s="54" t="inlineStr">
+        <is>
+          <t>Monthly cohort revenue</t>
+        </is>
+      </c>
+      <c r="B22" s="56">
+        <f>B12*(B10+B11*'2_Pricing'!B19)</f>
+        <v/>
+      </c>
+      <c r="C22" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D22" s="54" t="inlineStr">
+        <is>
+          <t>derived forecast</t>
+        </is>
+      </c>
+      <c r="E22" s="54" t="inlineStr">
+        <is>
+          <t>Base is additional, no included-report double charge</t>
+        </is>
+      </c>
+      <c r="F22" s="54" t="inlineStr">
+        <is>
+          <t>Hybrid pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1" s="45">
+      <c r="A23" s="54" t="inlineStr">
+        <is>
+          <t>Blended cohort GM</t>
+        </is>
+      </c>
+      <c r="B23" s="56">
+        <f>1-B21/B22</f>
+        <v/>
+      </c>
+      <c r="C23" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D23" s="54" t="inlineStr">
+        <is>
+          <t>derived forecast</t>
+        </is>
+      </c>
+      <c r="E23" s="54" t="inlineStr">
+        <is>
+          <t>COGS includes workspace service; show separately from report GM</t>
+        </is>
+      </c>
+      <c r="F23" s="54" t="inlineStr">
+        <is>
+          <t>B21:B22</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" s="45">
+      <c r="A24" s="54" t="inlineStr">
+        <is>
+          <t>Fully loaded Cost/Job</t>
+        </is>
+      </c>
+      <c r="B24" s="56">
+        <f>'1_Cost_Job'!B67</f>
+        <v/>
+      </c>
+      <c r="C24" s="54" t="inlineStr">
+        <is>
+          <t>USD/report</t>
+        </is>
+      </c>
+      <c r="D24" s="54" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E24" s="54" t="inlineStr">
+        <is>
+          <t>Overhead not included in gross margin</t>
+        </is>
+      </c>
+      <c r="F24" s="54" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B67</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" s="45">
+      <c r="A25" s="54" t="inlineStr">
+        <is>
+          <t>ARPU</t>
+        </is>
+      </c>
+      <c r="B25" s="56">
+        <f>B10+B11*'2_Pricing'!B19</f>
+        <v/>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D25" s="54" t="inlineStr">
+        <is>
+          <t>derived forecast</t>
+        </is>
+      </c>
+      <c r="E25" s="54" t="inlineStr">
+        <is>
+          <t>39 base + 3×60 reports</t>
+        </is>
+      </c>
+      <c r="F25" s="54" t="inlineStr">
+        <is>
+          <t>B10:B11</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" s="45">
+      <c r="A26" s="54" t="inlineStr">
+        <is>
+          <t>Conservative channel GM</t>
+        </is>
+      </c>
+      <c r="B26" s="56">
+        <f>'2_Pricing'!B21</f>
+        <v/>
+      </c>
+      <c r="C26" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D26" s="54" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E26" s="54" t="inlineStr">
+        <is>
+          <t>Use report GM, lower than blended; conservative CAC cap</t>
+        </is>
+      </c>
+      <c r="F26" s="54" t="inlineStr">
+        <is>
+          <t>2_Pricing!B21</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" s="45">
+      <c r="A27" s="54" t="inlineStr">
+        <is>
+          <t>CAC budget</t>
+        </is>
+      </c>
+      <c r="B27" s="56">
+        <f>'4_Channel_Fit'!B9</f>
+        <v/>
+      </c>
+      <c r="C27" s="54" t="inlineStr">
+        <is>
+          <t>USD/customer</t>
+        </is>
+      </c>
+      <c r="D27" s="54" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E27" s="54" t="inlineStr">
+        <is>
+          <t>SMB 12-month ceiling is lab convention, not proved retention</t>
+        </is>
+      </c>
+      <c r="F27" s="54" t="inlineStr">
+        <is>
+          <t>4_Channel_Fit!B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" s="45">
+      <c r="A28" s="54" t="inlineStr">
+        <is>
+          <t>PLG acquisition spend</t>
+        </is>
+      </c>
+      <c r="B28" s="55" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C28" s="54" t="inlineStr">
+        <is>
+          <t>USD/90days</t>
+        </is>
+      </c>
+      <c r="D28" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E28" s="54" t="inlineStr">
+        <is>
+          <t>$800 founder content (40h×$20) + $200 content tools + $200 placement</t>
+        </is>
+      </c>
+      <c r="F28" s="54" t="inlineStr">
+        <is>
+          <t>No actual spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" s="45">
+      <c r="A29" s="54" t="inlineStr">
+        <is>
+          <t>GitHub App installs</t>
+        </is>
+      </c>
+      <c r="B29" s="55" t="n">
+        <v>60</v>
+      </c>
+      <c r="C29" s="54" t="inlineStr">
+        <is>
+          <t>installs/90days</t>
+        </is>
+      </c>
+      <c r="D29" s="54" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E29" s="54" t="inlineStr">
+        <is>
+          <t>Qualified org installations, not pageviews</t>
+        </is>
+      </c>
+      <c r="F29" s="54" t="inlineStr">
+        <is>
+          <t>No actual installs</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" s="45">
+      <c r="A30" s="54" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="B30" s="55" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C30" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D30" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E30" s="54" t="inlineStr">
+        <is>
+          <t>First AI-ready report within 14 days</t>
+        </is>
+      </c>
+      <c r="F30" s="54" t="inlineStr">
+        <is>
+          <t>Pilot funnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" s="45">
+      <c r="A31" s="54" t="inlineStr">
+        <is>
+          <t>Activation to paid</t>
+        </is>
+      </c>
+      <c r="B31" s="55" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C31" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D31" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E31" s="54" t="inlineStr">
+        <is>
+          <t>3 paid from 12 activated</t>
+        </is>
+      </c>
+      <c r="F31" s="54" t="inlineStr">
+        <is>
+          <t>Pilot funnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" s="45">
+      <c r="A32" s="54" t="inlineStr">
+        <is>
+          <t>PLG paid customers</t>
+        </is>
+      </c>
+      <c r="B32" s="56">
+        <f>B29*B30*B31</f>
+        <v/>
+      </c>
+      <c r="C32" s="54" t="inlineStr">
+        <is>
+          <t>customers</t>
+        </is>
+      </c>
+      <c r="D32" s="54" t="inlineStr">
+        <is>
+          <t>derived target</t>
+        </is>
+      </c>
+      <c r="E32" s="54" t="inlineStr">
+        <is>
+          <t>No sales rep or partner commission</t>
+        </is>
+      </c>
+      <c r="F32" s="54" t="inlineStr">
+        <is>
+          <t>B29:B31</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1" s="45">
+      <c r="A33" s="54" t="inlineStr">
+        <is>
+          <t>PLG CAC</t>
+        </is>
+      </c>
+      <c r="B33" s="56">
+        <f>B28/B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="54" t="inlineStr">
+        <is>
+          <t>USD/customer</t>
+        </is>
+      </c>
+      <c r="D33" s="54" t="inlineStr">
+        <is>
+          <t>derived estimate</t>
+        </is>
+      </c>
+      <c r="E33" s="54" t="inlineStr">
+        <is>
+          <t>Includes founder time and free trial service allowance</t>
+        </is>
+      </c>
+      <c r="F33" s="54" t="inlineStr">
+        <is>
+          <t>B28:B32</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" s="45">
+      <c r="A34" s="54" t="inlineStr">
+        <is>
+          <t>PLG payback months</t>
+        </is>
+      </c>
+      <c r="B34" s="56">
+        <f>B33/('4_Channel_Fit'!B5*'4_Channel_Fit'!B6)</f>
+        <v/>
+      </c>
+      <c r="C34" s="54" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D34" s="54" t="inlineStr">
+        <is>
+          <t>derived estimate</t>
+        </is>
+      </c>
+      <c r="E34" s="54" t="inlineStr">
+        <is>
+          <t>Use conservative report GM</t>
+        </is>
+      </c>
+      <c r="F34" s="54" t="inlineStr">
+        <is>
+          <t>4_Channel_Fit!B5:B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1" s="45">
+      <c r="A35" s="54" t="inlineStr">
+        <is>
+          <t>PLG operating CAC stop threshold</t>
+        </is>
+      </c>
+      <c r="B35" s="55" t="n">
+        <v>400</v>
+      </c>
+      <c r="C35" s="54" t="inlineStr">
+        <is>
+          <t>USD/customer</t>
+        </is>
+      </c>
+      <c r="D35" s="54" t="inlineStr">
+        <is>
+          <t>decision hypothesis</t>
+        </is>
+      </c>
+      <c r="E35" s="54" t="inlineStr">
+        <is>
+          <t>Pause paid acquisition above $400 until conversion measured</t>
+        </is>
+      </c>
+      <c r="F35" s="54" t="inlineStr">
+        <is>
+          <t>PLG plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1" s="45">
+      <c r="A36" s="54" t="inlineStr">
+        <is>
+          <t>Shared service monthly floor</t>
+        </is>
+      </c>
+      <c r="B36" s="55" t="n">
+        <v>80</v>
+      </c>
+      <c r="C36" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D36" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E36" s="54" t="inlineStr">
+        <is>
+          <t>Hosting, auth and connectors minimum; requires invoice</t>
+        </is>
+      </c>
+      <c r="F36" s="54" t="inlineStr">
+        <is>
+          <t>Infra estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" s="45">
+      <c r="A37" s="54" t="inlineStr">
+        <is>
+          <t>Infra variable/attempt</t>
+        </is>
+      </c>
+      <c r="B37" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" s="54" t="inlineStr">
+        <is>
+          <t>USD/attempt</t>
+        </is>
+      </c>
+      <c r="D37" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E37" s="54" t="inlineStr">
+        <is>
+          <t>$3 ingestion/DB + $1 storage/egress + $1 logging/eval + $1.5 support + $1.5 collection/reserve</t>
+        </is>
+      </c>
+      <c r="F37" s="54" t="inlineStr">
+        <is>
+          <t>Infra estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1" s="45">
+      <c r="A38" s="54" t="inlineStr">
+        <is>
+          <t>Vendor QA minutes</t>
+        </is>
+      </c>
+      <c r="B38" s="56">
+        <f>'1_Cost_Job'!B52</f>
+        <v/>
+      </c>
+      <c r="C38" s="54" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="D38" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E38" s="54" t="inlineStr">
+        <is>
+          <t>Early sample review of evidence links and numerical accuracy</t>
+        </is>
+      </c>
+      <c r="F38" s="54" t="inlineStr">
+        <is>
+          <t>QA plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1" s="45">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>Vendor fully loaded hourly rate</t>
+        </is>
+      </c>
+      <c r="B39" s="56">
+        <f>'1_Cost_Job'!B50</f>
+        <v/>
+      </c>
+      <c r="C39" s="54" t="inlineStr">
+        <is>
+          <t>USD/hour</t>
+        </is>
+      </c>
+      <c r="D39" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E39" s="54" t="inlineStr">
+        <is>
+          <t>Labor estimate including burden</t>
+        </is>
+      </c>
+      <c r="F39" s="54" t="inlineStr">
+        <is>
+          <t>QA plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1" s="45">
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <t>Rep motion total annual acquisition cost</t>
+        </is>
+      </c>
+      <c r="B40" s="55" t="n">
+        <v>48000</v>
+      </c>
+      <c r="C40" s="54" t="inlineStr">
+        <is>
+          <t>USD/year</t>
+        </is>
+      </c>
+      <c r="D40" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E40" s="54" t="inlineStr">
+        <is>
+          <t>$24k AE + $12k marketing + $12k tools/management; fully loaded, local scenario</t>
+        </is>
+      </c>
+      <c r="F40" s="54" t="inlineStr">
+        <is>
+          <t>Not ICONIQ benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1" s="45">
+      <c r="A41" s="54" t="inlineStr">
+        <is>
+          <t>Rep qualified opportunities/year</t>
+        </is>
+      </c>
+      <c r="B41" s="55" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t>opportunities</t>
+        </is>
+      </c>
+      <c r="D41" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E41" s="54" t="inlineStr">
+        <is>
+          <t>Low-velocity technical approval; replaces unknown external CPO</t>
+        </is>
+      </c>
+      <c r="F41" s="54" t="inlineStr">
+        <is>
+          <t>Local scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1" s="45">
+      <c r="A42" s="54" t="inlineStr">
+        <is>
+          <t>Rep cost/opportunity</t>
+        </is>
+      </c>
+      <c r="B42" s="56">
+        <f>B40/B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="54" t="inlineStr">
+        <is>
+          <t>USD/opportunity</t>
+        </is>
+      </c>
+      <c r="D42" s="54" t="inlineStr">
+        <is>
+          <t>derived estimate</t>
+        </is>
+      </c>
+      <c r="E42" s="54" t="inlineStr">
+        <is>
+          <t>Full acquisition cost divided by qualified opportunities</t>
+        </is>
+      </c>
+      <c r="F42" s="54" t="inlineStr">
+        <is>
+          <t>B40:B41</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1" s="45">
+      <c r="A43" s="54" t="inlineStr">
+        <is>
+          <t>Rep win rate</t>
+        </is>
+      </c>
+      <c r="B43" s="55" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C43" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D43" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E43" s="54" t="inlineStr">
+        <is>
+          <t>10 wins from 40 opportunities</t>
+        </is>
+      </c>
+      <c r="F43" s="54" t="inlineStr">
+        <is>
+          <t>Local scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1" s="45">
+      <c r="A44" s="54" t="inlineStr">
+        <is>
+          <t>Rep CAC</t>
+        </is>
+      </c>
+      <c r="B44" s="56">
+        <f>B42/B43</f>
+        <v/>
+      </c>
+      <c r="C44" s="54" t="inlineStr">
+        <is>
+          <t>USD/customer</t>
+        </is>
+      </c>
+      <c r="D44" s="54" t="inlineStr">
+        <is>
+          <t>derived estimate</t>
+        </is>
+      </c>
+      <c r="E44" s="54" t="inlineStr">
+        <is>
+          <t>Not measured or third-party industry statistic</t>
+        </is>
+      </c>
+      <c r="F44" s="54" t="inlineStr">
+        <is>
+          <t>B42:B43</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1" s="45">
+      <c r="A45" s="54" t="inlineStr">
+        <is>
+          <t>AE annual quota</t>
+        </is>
+      </c>
+      <c r="B45" s="55" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C45" s="54" t="inlineStr">
+        <is>
+          <t>USD/year</t>
+        </is>
+      </c>
+      <c r="D45" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E45" s="54" t="inlineStr">
+        <is>
+          <t>5× $24k fully loaded cost; conventional planning ratio, not benchmark</t>
+        </is>
+      </c>
+      <c r="F45" s="54" t="inlineStr">
+        <is>
+          <t>Sales scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="48" customHeight="1" s="45">
+      <c r="A46" s="54" t="inlineStr">
+        <is>
+          <t>AE annual fully loaded cost</t>
+        </is>
+      </c>
+      <c r="B46" s="55" t="n">
+        <v>24000</v>
+      </c>
+      <c r="C46" s="54" t="inlineStr">
+        <is>
+          <t>USD/year</t>
+        </is>
+      </c>
+      <c r="D46" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E46" s="54" t="inlineStr">
+        <is>
+          <t>$2,000/month inclusive burden; not actual payroll</t>
+        </is>
+      </c>
+      <c r="F46" s="54" t="inlineStr">
+        <is>
+          <t>Sales scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1" s="45">
+      <c r="A47" s="54" t="inlineStr">
+        <is>
+          <t>Working days/year</t>
+        </is>
+      </c>
+      <c r="B47" s="55" t="n">
+        <v>250</v>
+      </c>
+      <c r="C47" s="54" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D47" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E47" s="54" t="inlineStr">
+        <is>
+          <t>Lab working-year assumption</t>
+        </is>
+      </c>
+      <c r="F47" s="54" t="inlineStr">
+        <is>
+          <t>Channel inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1" s="45">
+      <c r="A48" s="54" t="inlineStr">
+        <is>
+          <t>Total value-based monthly ceiling</t>
+        </is>
+      </c>
+      <c r="B48" s="56">
+        <f>'2_Pricing'!B10*0.25</f>
+        <v/>
+      </c>
+      <c r="C48" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D48" s="54" t="inlineStr">
+        <is>
+          <t>derived hypothesis</t>
+        </is>
+      </c>
+      <c r="E48" s="54" t="inlineStr">
+        <is>
+          <t>25% of value; all-in bill must fit, including base fee</t>
+        </is>
+      </c>
+      <c r="F48" s="54" t="inlineStr">
+        <is>
+          <t>2_Pricing!B10</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="48" customHeight="1" s="45">
+      <c r="A49" s="54" t="inlineStr">
+        <is>
+          <t>Overhead/month</t>
+        </is>
+      </c>
+      <c r="B49" s="56">
+        <f>'1_Cost_Job'!B59</f>
+        <v/>
+      </c>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D49" s="54" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="E49" s="54" t="inlineStr">
+        <is>
+          <t>Product upkeep and admin, excludes CAC and direct support</t>
+        </is>
+      </c>
+      <c r="F49" s="54" t="inlineStr">
+        <is>
+          <t>1_Cost_Job!B59</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="48" customHeight="1" s="45">
+      <c r="A50" s="54" t="inlineStr">
+        <is>
+          <t>All-in baseline customer bill</t>
+        </is>
+      </c>
+      <c r="B50" s="56">
+        <f>B25</f>
+        <v/>
+      </c>
+      <c r="C50" s="54" t="inlineStr">
+        <is>
+          <t>USD/month</t>
+        </is>
+      </c>
+      <c r="D50" s="54" t="inlineStr">
+        <is>
+          <t>pricing hypothesis</t>
+        </is>
+      </c>
+      <c r="E50" s="54" t="inlineStr">
+        <is>
+          <t>Opt-in before overage; no auto unlimited retries</t>
+        </is>
+      </c>
+      <c r="F50" s="54" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="48" customHeight="1" s="45">
+      <c r="A51" s="54" t="inlineStr">
+        <is>
+          <t>USD/VND sell quote</t>
+        </is>
+      </c>
+      <c r="B51" s="56">
+        <f>'1_Cost_Job'!B68</f>
+        <v/>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t>VND/USD</t>
+        </is>
+      </c>
+      <c r="D51" s="54" t="inlineStr">
+        <is>
+          <t>verified 2026-10-08</t>
+        </is>
+      </c>
+      <c r="E51" s="54" t="inlineStr">
+        <is>
+          <t>VCB XML published 12:13:07 PM</t>
+        </is>
+      </c>
+      <c r="F51" s="54" t="inlineStr">
+        <is>
+          <t>data/sources.json#vietcombank</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="48" customHeight="1" s="45">
+      <c r="A52" s="54" t="inlineStr">
+        <is>
+          <t>Price/source check date</t>
+        </is>
+      </c>
+      <c r="B52" s="55" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C52" s="54" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D52" s="54" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="E52" s="54" t="inlineStr">
+        <is>
+          <t>Chosen vendor and peers; not all historical rows</t>
+        </is>
+      </c>
+      <c r="F52" s="54" t="inlineStr">
+        <is>
+          <t>data/sources.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="48" customHeight="1" s="45">
+      <c r="A53" s="54" t="inlineStr">
+        <is>
+          <t>GM50 containment threshold</t>
+        </is>
+      </c>
+      <c r="B53" s="56">
+        <f>('2_Pricing'!B29+'2_Pricing'!B30)/('2_Pricing'!B19*0.5)</f>
+        <v/>
+      </c>
+      <c r="C53" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D53" s="54" t="inlineStr">
+        <is>
+          <t>derived A-only</t>
+        </is>
+      </c>
+      <c r="E53" s="54" t="inlineStr">
+        <is>
+          <t>Below this threshold report GM &lt;50%</t>
+        </is>
+      </c>
+      <c r="F53" s="54" t="inlineStr">
+        <is>
+          <t>2_Pricing!B29:B30</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="48" customHeight="1" s="45">
+      <c r="A54" s="54" t="inlineStr">
+        <is>
+          <t>GM60 containment threshold</t>
+        </is>
+      </c>
+      <c r="B54" s="56">
+        <f>'2_Pricing'!B33</f>
+        <v/>
+      </c>
+      <c r="C54" s="54" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D54" s="54" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E54" s="54" t="inlineStr">
+        <is>
+          <t>Not accounting breakeven GM=0; healthy-margin floor</t>
+        </is>
+      </c>
+      <c r="F54" s="54" t="inlineStr">
+        <is>
+          <t>2_Pricing!B33</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="48" customHeight="1" s="45">
+      <c r="A55" s="54" t="inlineStr">
+        <is>
+          <t>Monthly report cadence</t>
+        </is>
+      </c>
+      <c r="B55" s="55" t="inlineStr">
+        <is>
+          <t>2 Sprint + 1 Board</t>
+        </is>
+      </c>
+      <c r="C55" s="54" t="inlineStr">
+        <is>
+          <t>reports/month</t>
+        </is>
+      </c>
+      <c r="D55" s="54" t="inlineStr">
+        <is>
+          <t>Day20 target</t>
+        </is>
+      </c>
+      <c r="E55" s="54" t="inlineStr">
+        <is>
+          <t>Mean completed preparation jobs =3/workspace</t>
+        </is>
+      </c>
+      <c r="F55" s="54" t="inlineStr">
+        <is>
+          <t>Day20 engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="48" customHeight="1" s="45">
+      <c r="A56" s="54" t="inlineStr">
+        <is>
+          <t>Trial/activation window</t>
+        </is>
+      </c>
+      <c r="B56" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="C56" s="54" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D56" s="54" t="inlineStr">
+        <is>
+          <t>design target</t>
+        </is>
+      </c>
+      <c r="E56" s="54" t="inlineStr">
+        <is>
+          <t>One small redacted report; no unlimited full-history trial</t>
+        </is>
+      </c>
+      <c r="F56" s="54" t="inlineStr">
+        <is>
+          <t>Day20 activation</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="48" customHeight="1" s="45">
+      <c r="A57" s="54" t="inlineStr">
+        <is>
+          <t>Attempt quota/workspace/month</t>
+        </is>
+      </c>
+      <c r="B57" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="C57" s="54" t="inlineStr">
+        <is>
+          <t>attempts</t>
+        </is>
+      </c>
+      <c r="D57" s="54" t="inlineStr">
+        <is>
+          <t>design proposal</t>
+        </is>
+      </c>
+      <c r="E57" s="54" t="inlineStr">
+        <is>
+          <t>Alerts then pause; user approves revised quota/price</t>
+        </is>
+      </c>
+      <c r="F57" s="54" t="inlineStr">
+        <is>
+          <t>Usage guardrail</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="48" customHeight="1" s="45">
+      <c r="A58" s="54" t="inlineStr">
+        <is>
+          <t>Dataset PR limit/workspace/month</t>
+        </is>
+      </c>
+      <c r="B58" s="55" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C58" s="54" t="inlineStr">
+        <is>
+          <t>PR metadata records</t>
+        </is>
+      </c>
+      <c r="D58" s="54" t="inlineStr">
+        <is>
+          <t>design proposal</t>
+        </is>
+      </c>
+      <c r="E58" s="54" t="inlineStr">
+        <is>
+          <t>Beyond limit: no silent ingestion or overage</t>
+        </is>
+      </c>
+      <c r="F58" s="54" t="inlineStr">
+        <is>
+          <t>Usage guardrail</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="48" customHeight="1" s="45">
+      <c r="A59" s="54" t="inlineStr">
+        <is>
+          <t>Raw metadata retention</t>
+        </is>
+      </c>
+      <c r="B59" s="55" t="n">
+        <v>90</v>
+      </c>
+      <c r="C59" s="54" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D59" s="54" t="inlineStr">
+        <is>
+          <t>policy proposal</t>
+        </is>
+      </c>
+      <c r="E59" s="54" t="inlineStr">
+        <is>
+          <t>Must verify export/deletion before pilot; not implemented claim</t>
+        </is>
+      </c>
+      <c r="F59" s="54" t="inlineStr">
+        <is>
+          <t>Procurement Q&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="48" customHeight="1" s="45">
+      <c r="A60" s="54" t="inlineStr">
+        <is>
+          <t>Pilot orgs</t>
+        </is>
+      </c>
+      <c r="B60" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" s="54" t="inlineStr">
+        <is>
+          <t>organizations</t>
+        </is>
+      </c>
+      <c r="D60" s="54" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E60" s="54" t="inlineStr">
+        <is>
+          <t>Candidates not named yet; recruit voluntarily via PLG</t>
+        </is>
+      </c>
+      <c r="F60" s="54" t="inlineStr">
+        <is>
+          <t>5_90Day_Plan!B13</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="48" customHeight="1" s="45">
+      <c r="A61" s="54" t="inlineStr">
+        <is>
+          <t>Pilot duration</t>
+        </is>
+      </c>
+      <c r="B61" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" s="54" t="inlineStr">
+        <is>
+          <t>weeks</t>
+        </is>
+      </c>
+      <c r="D61" s="54" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E61" s="54" t="inlineStr">
+        <is>
+          <t>Not a completed pilot report</t>
+        </is>
+      </c>
+      <c r="F61" s="54" t="inlineStr">
+        <is>
+          <t>Pilot Protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="48" customHeight="1" s="45">
+      <c r="A62" s="54" t="inlineStr">
+        <is>
+          <t>Eval cases</t>
+        </is>
+      </c>
+      <c r="B62" s="55" t="n">
+        <v>100</v>
+      </c>
+      <c r="C62" s="54" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="D62" s="54" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E62" s="54" t="inlineStr">
+        <is>
+          <t>Stratified normal/edge/error reports; no eval result claim</t>
+        </is>
+      </c>
+      <c r="F62" s="54" t="inlineStr">
+        <is>
+          <t>Eval Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="48" customHeight="1" s="45">
+      <c r="A63" s="54" t="inlineStr">
+        <is>
+          <t>Eval due</t>
+        </is>
+      </c>
+      <c r="B63" s="55" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C63" s="54" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D63" s="54" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="E63" s="54" t="inlineStr">
+        <is>
+          <t>Owner Phạm Thanh Đạt</t>
+        </is>
+      </c>
+      <c r="F63" s="54" t="inlineStr">
+        <is>
+          <t>5_90Day_Plan!D23</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="48" customHeight="1" s="45">
+      <c r="A64" s="54" t="inlineStr">
+        <is>
+          <t>Procurement control verification due</t>
+        </is>
+      </c>
+      <c r="B64" s="55" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C64" s="54" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D64" s="54" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="E64" s="54" t="inlineStr">
+        <is>
+          <t>Written answers drafted; live proof pending</t>
+        </is>
+      </c>
+      <c r="F64" s="54" t="inlineStr">
+        <is>
+          <t>5_90Day_Plan!D24</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="48" customHeight="1" s="45">
+      <c r="A65" s="54" t="inlineStr">
+        <is>
+          <t>Pilot report due</t>
+        </is>
+      </c>
+      <c r="B65" s="55" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="C65" s="54" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D65" s="54" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="E65" s="54" t="inlineStr">
+        <is>
+          <t>Recruitment/consent and measured logs required</t>
+        </is>
+      </c>
+      <c r="F65" s="54" t="inlineStr">
+        <is>
+          <t>5_90Day_Plan!D25</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="48" customHeight="1" s="45">
+      <c r="A66" s="54" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="B66" s="55" t="inlineStr">
+        <is>
+          <t>Phạm Thanh Đạt</t>
+        </is>
+      </c>
+      <c r="C66" s="54" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D66" s="54" t="inlineStr">
+        <is>
+          <t>assignment</t>
+        </is>
+      </c>
+      <c r="E66" s="54" t="inlineStr">
+        <is>
+          <t>Only named owner from input; no invented teammates</t>
+        </is>
+      </c>
+      <c r="F66" s="54" t="inlineStr">
+        <is>
+          <t>User submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="48" customHeight="1" s="45">
+      <c r="A67" s="54" t="inlineStr">
+        <is>
+          <t>Independent human reader test</t>
+        </is>
+      </c>
+      <c r="B67" s="55" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="C67" s="54" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D67" s="54" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E67" s="54" t="inlineStr">
+        <is>
+          <t>AI review cannot substitute an actual stranger</t>
+        </is>
+      </c>
+      <c r="F67" s="54" t="inlineStr">
+        <is>
+          <t>5_90Day_Plan!B29:B32</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="48" customHeight="1" s="45">
+      <c r="A68" s="54" t="inlineStr">
+        <is>
+          <t>Historical template benchmark scope</t>
+        </is>
+      </c>
+      <c r="B68" s="55" t="inlineStr">
+        <is>
+          <t>Chỉ Haiku/cache đã kiểm tra; các dòng khác giữ nguyên tham chiếu cũ</t>
+        </is>
+      </c>
+      <c r="C68" s="54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D68" s="54" t="inlineStr">
+        <is>
+          <t>not verified current</t>
+        </is>
+      </c>
+      <c r="E68" s="54" t="inlineStr">
+        <is>
+          <t>No use of unverified promotional or ICONIQ prices</t>
+        </is>
+      </c>
+      <c r="F68" s="54" t="inlineStr">
+        <is>
+          <t>6_Benchmarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="48" customHeight="1" s="45">
+      <c r="A69" s="54" t="inlineStr">
+        <is>
+          <t>Planned end-of-90days model accounts</t>
+        </is>
+      </c>
+      <c r="B69" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="C69" s="54" t="inlineStr">
+        <is>
+          <t>workspaces</t>
+        </is>
+      </c>
+      <c r="D69" s="54" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E69" s="54" t="inlineStr">
+        <is>
+          <t>Not same as 3 incremental funnel wins; pilot+repeat funnel cohorts required</t>
+        </is>
+      </c>
+      <c r="F69" s="54" t="inlineStr">
+        <is>
+          <t>90-day plan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F3"/>
+  <autoFilter ref="A3:F69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(cp4): choose PLG with bottom-up CAC affordability
</commit_message>
<xml_diff>
--- a/deliverables/Day22-DevPulse-Monetization-Model.xlsx
+++ b/deliverables/Day22-DevPulse-Monetization-Model.xlsx
@@ -522,6 +522,46 @@
 </file>
 
 <file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Day22 provenance</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>39 base + 3 AI-ready reports ×60 =219 USD/month. Expected ARPU, not current revenue.</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>SMB engineering team20–50 devs, per Day20. 12-month payback is lab ceiling, not retention evidence; use tighter CAC $400 operating stop.</t>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0">
+      <text>
+        <t>Local planning quota120k/year =5×24k fully loaded AE cost. Not historical $500k quota copied from Tunguz.</t>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0" shapeId="0">
+      <text>
+        <t>Local bottom-up scenario: 48k annual rep motion acquisition spend /40 qualified opportunities =1200. Not unverified ICONIQ2026 cost-per-opportunity.</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0">
+      <text>
+        <t>25% assumption:10 wins/40 opportunities; replace with actual funnel.</t>
+      </text>
+    </comment>
+    <comment ref="B38" authorId="0" shapeId="0">
+      <text>
+        <t>PLG is a proposed 90-day motion, not a functioning current acquisition channel. GitHub App installation and trust friction are principal falsification risks.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Day22 provenance</author>
@@ -6852,8 +6892,8 @@
           <t>ARPU / tháng ($)</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n">
-        <v>200</v>
+      <c r="B5" s="53" t="n">
+        <v>219</v>
       </c>
     </row>
     <row r="6">
@@ -6867,13 +6907,13 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="32" customHeight="1" s="45">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Phân khúc (SMB / Mid / Enterprise)</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>SMB</t>
         </is>
@@ -6947,8 +6987,8 @@
           <t>Quota / AE / năm ($)</t>
         </is>
       </c>
-      <c r="B13" s="25" t="n">
-        <v>500000</v>
+      <c r="B13" s="53" t="n">
+        <v>120000</v>
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
@@ -6962,7 +7002,7 @@
           <t>Số ngày làm việc / năm</t>
         </is>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="48" t="n">
         <v>250</v>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -7029,8 +7069,8 @@
           <t>Cost per opportunity ($)</t>
         </is>
       </c>
-      <c r="B20" s="25" t="n">
-        <v>8000</v>
+      <c r="B20" s="53" t="n">
+        <v>1200</v>
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
@@ -7044,7 +7084,7 @@
           <t>Win rate</t>
         </is>
       </c>
-      <c r="B21" s="16" t="n">
+      <c r="B21" s="49" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -7129,14 +7169,14 @@
           <t>1. Ngân sách CAC của tôi nuôi nổi kênh này</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" s="13" t="n">
-        <v>3</v>
+      <c r="B28" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="47" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="45">
@@ -7145,14 +7185,14 @@
           <t>2. Khách hàng mục tiêu thực sự mua theo cách này</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n">
+      <c r="B29" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" s="13" t="n">
-        <v>3</v>
+      <c r="C29" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="47" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="45">
@@ -7161,14 +7201,14 @@
           <t>3. Đội hiện tại có năng lực chạy kênh này ngay</t>
         </is>
       </c>
-      <c r="B30" s="13" t="n">
+      <c r="B30" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="C30" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <v>3</v>
+      <c r="C30" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="47" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="45">
@@ -7177,14 +7217,14 @@
           <t>4. Tôi tiếp cận được điểm nhúng / partner trong 30 ngày</t>
         </is>
       </c>
-      <c r="B31" s="13" t="n">
+      <c r="B31" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="C31" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>3</v>
+      <c r="C31" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="47" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="45">
@@ -7193,13 +7233,13 @@
           <t>5. Kênh này đưa tôi đến ĐÚNG Pain Moment</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="C32" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D32" s="13" t="n">
+      <c r="D32" s="47" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7209,14 +7249,14 @@
           <t>6. Tôi đo được hiệu quả trong vòng 90 ngày</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="C33" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <v>3</v>
+      <c r="D33" s="47" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="45">
@@ -7264,15 +7304,15 @@
       <c r="G37" s="10" t="n"/>
       <c r="H37" s="10" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="45">
+    <row r="38" ht="32" customHeight="1" s="45">
       <c r="A38" s="14" t="inlineStr">
         <is>
           <t>★ Kênh tôi chọn cho 90 ngày đầu</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Partner-Led</t>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>PLG</t>
         </is>
       </c>
       <c r="D38" s="17" t="inlineStr">
@@ -7281,46 +7321,58 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1" s="45">
+    <row r="39" ht="46.25" customHeight="1" s="45">
       <c r="A39" s="14" t="inlineStr">
         <is>
           <t>Nếu Partner-Led: TÊN CÔNG TY partner</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n"/>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>Không áp dụng: GitHub, Inc. là bề mặt phân phối, chưa có partner hợp đồng.</t>
+        </is>
+      </c>
       <c r="D39" s="17" t="inlineStr">
         <is>
           <t>'Các nền tảng trong ngành' = chưa có kênh</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1" s="45">
+    <row r="40" ht="32" customHeight="1" s="45">
       <c r="A40" s="14" t="inlineStr">
         <is>
           <t>Đã nói chuyện với họ chưa? (Rồi / Chưa)</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Chưa</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1" s="45">
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>Chưa; không chọn Partner-Led</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="51.25" customHeight="1" s="45">
       <c r="A41" s="14" t="inlineStr">
         <is>
           <t>Bạn mang lại giá trị gì cho partner?</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1" s="45">
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>Không áp dụng. Khách tự cài GitHub App; không giả quan hệ partner hoặc commission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60.625" customHeight="1" s="45">
       <c r="A42" s="14" t="inlineStr">
         <is>
           <t>Nếu rơi vào vùng không khả thi — lối thoát nào?</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n"/>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>Giữ PLG tự phục vụ; thử 3 pilot nhỏ trong 30 ngày. Không tuyển AE khi CAC rep $4.800 vượt budget.</t>
+        </is>
+      </c>
       <c r="D42" s="17" t="inlineStr">
         <is>
           <t>Giảm giá để tự phục vụ / tăng giá + service / Partner-Led</t>
@@ -8293,6 +8345,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs(cp6): deliver traced one-pager and honest evidence pack
</commit_message>
<xml_diff>
--- a/deliverables/Day22-DevPulse-Monetization-Model.xlsx
+++ b/deliverables/Day22-DevPulse-Monetization-Model.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Assumptions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7_Assumptions'!$A$3:$F$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7_Assumptions'!$A$3:$F$90</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -5779,7 +5779,7 @@
       </ns0:c>
       <ns0:c r="C27" s="46" t="inlineStr">
         <ns0:is>
-          <ns0:t>$29/user/tháng annual; 1.000 credits; thêm từ $0,015/credit</ns0:t>
+          <ns0:t>$29/user/tháng annual; ≥50 dev; 1.000 credits; thêm từ $0,015/credit</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D27" s="46" t="inlineStr">
@@ -8506,7 +8506,7 @@
         </ns0:is>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="13" ht="68.75" customHeight="1" s="45">
+    <ns0:row r="13" ht="91.25" customHeight="1" s="45">
       <ns0:c r="A13" s="14" t="inlineStr">
         <ns0:is>
           <ns0:t>Mục tiêu số khách</ns0:t>
@@ -8519,12 +8519,12 @@
       </ns0:c>
       <ns0:c r="C13" s="46" t="inlineStr">
         <ns0:is>
-          <ns0:t>60 qualified installs; 12 activation; 3 paid; 10 active workspaces mục tiêu, không đồng nghĩa 10 paid</ns0:t>
+          <ns0:t>60 qualified installs; 12 activation; 3 paid. 10 paying workspace chỉ là steady-state scenario sau cohort đầu.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D13" s="46" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chưa cam kết số khách mới; chỉ scale sau gate; đủ ≥4 paid trước giá steady-state $60 với shared floor hiện tại</ns0:t>
+          <ns0:t>Chưa cam kết khách mới; ≥4 serviced paid chỉ là minimum theo c=75% planning; rollout phải đạt floor3× và GM60 bằng eval lower bound ở volume thật.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -11824,7 +11824,7 @@
     <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
     <ns0:pageSetUpPr fitToPage="1"/>
   </ns0:sheetPr>
-  <ns0:dimension ref="A1:F78"/>
+  <ns0:dimension ref="A1:F90"/>
   <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <ns0:cols>
     <ns0:col width="30" customWidth="1" style="45" min="1" max="1"/>
@@ -12652,7 +12652,7 @@
       </ns0:c>
       <ns0:c r="E28" s="54" t="inlineStr">
         <ns0:is>
-          <ns0:t>$800 founder content (40h×$20) + $200 content tools + $200 placement</ns0:t>
+          <ns0:t>$800 founder40h×20 + $200 tools + $200 placement/trial ($150 trial variable reserve + $50 placement). Not actual spend.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F28" s="54" t="inlineStr">
@@ -13893,7 +13893,7 @@
     <ns0:row r="69" ht="48" customHeight="1" s="45">
       <ns0:c r="A69" s="54" t="inlineStr">
         <ns0:is>
-          <ns0:t>90-day active workspace target</ns0:t>
+          <ns0:t>Later steady-state paid scenario</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="B69" s="55" t="n">
@@ -13911,7 +13911,7 @@
       </ns0:c>
       <ns0:c r="E69" s="54" t="inlineStr">
         <ns0:is>
-          <ns0:t>10 active, not all paid. Baseline10 paying is steady-state scenario beyond initial funnel.</ns0:t>
+          <ns0:t>Not Day90 target. Initial funnel3paid; do not continuously serve7unpaid tenants with paying-cohort economics.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F69" s="54" t="inlineStr">
@@ -14153,12 +14153,12 @@
       </ns0:c>
       <ns0:c r="D77" s="54" t="inlineStr">
         <ns0:is>
-          <ns0:t>derived rounded condition</ns0:t>
+          <ns0:t>point-estimate planning</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E77" s="54" t="inlineStr">
         <ns0:is>
-          <ns0:t>40-attempt baseline assumes10paid; at4paid/16attempts floor&lt;$60</ns0:t>
+          <ns0:t>Only4serviced paying orgs at75% point estimate; full rollout must verify floor3× and GM60 at eval lower bound and actual volume.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F77" s="54" t="inlineStr">
@@ -14198,8 +14198,376 @@
         </ns0:is>
       </ns0:c>
     </ns0:row>
+    <ns0:row r="79" ht="48" customHeight="1" s="45">
+      <ns0:c r="A79" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PLG activated customers</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B79" s="56">
+        <ns0:f>B29*B30</ns0:f>
+        <ns0:v>12</ns0:v>
+      </ns0:c>
+      <ns0:c r="C79" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>organizations</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D79" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>derived target</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E79" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only activated users receive one bounded report, not all60installs</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F79" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PLG funnel</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="80" ht="48" customHeight="1" s="45">
+      <ns0:c r="A80" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Course day</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B80" s="55" t="n">
+        <ns0:v>22</ns0:v>
+      </ns0:c>
+      <ns0:c r="C80" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>day</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D80" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>course identifier</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E80" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Template source filenames Day22; original workbook contains Day28 typo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F80" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Uploaded course</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="81" ht="48" customHeight="1" s="45">
+      <ns0:c r="A81" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Student identifier</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B81" s="55" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2A202602721</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C81" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>identifier</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D81" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>provided</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E81" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Not a financial figure</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F81" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>User repository name</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="82" ht="48" customHeight="1" s="45">
+      <ns0:c r="A82" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Trial variable service reserve</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B82" s="55" t="n">
+        <ns0:v>150</ns0:v>
+      </ns0:c>
+      <ns0:c r="C82" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>USD/90days</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D82" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>budget estimate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E82" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Within$200 acquisition placement/trial budget, not production COGS duplicate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F82" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PLG budget</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="83" ht="48" customHeight="1" s="45">
+      <ns0:c r="A83" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Trial expected attempts</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B83" s="56">
+        <ns0:f>B79/'1_Cost_Job'!B10</ns0:f>
+        <ns0:v>16</ns0:v>
+      </ns0:c>
+      <ns0:c r="C83" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>attempts</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D83" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>derived estimate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E83" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>12activated jobs /75% success; cap spend, no unlimited histories</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F83" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PLG forecast</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="84" ht="48" customHeight="1" s="45">
+      <ns0:c r="A84" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Trial variable COGS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B84" s="56">
+        <ns0:f>B83*(B37+'1_Cost_Job'!B31+'1_Cost_Job'!B38+'1_Cost_Job'!B47+'2_Pricing'!B30)</ns0:f>
+        <ns0:v>149.734912</ns0:v>
+      </ns0:c>
+      <ns0:c r="C84" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>USD/90days</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D84" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>derived estimate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E84" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sharedfloor80 assigned once to paid cohort; if no paid cohort, acquisition budget also bears floor</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F84" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PLG forecast</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="85" ht="48" customHeight="1" s="45">
+      <ns0:c r="A85" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pilot floor3x containment</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B85" s="56">
+        <ns0:f>B73*'1_Cost_Job'!B10*'2_Pricing'!B6/'2_Pricing'!B19</ns0:f>
+        <ns0:v>0.801254933333333</ns0:v>
+      </ns0:c>
+      <ns0:c r="C85" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>fraction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D85" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>derived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E85" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>3workspace requires80.12549% point containment for floor3x</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F85" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pilot scenario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="86" ht="48" customHeight="1" s="45">
+      <ns0:c r="A86" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Four-paid floor3x containment</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B86" s="56">
+        <ns0:f>((B36/(B77*B13))+B37+'1_Cost_Job'!B31+'1_Cost_Job'!B47+'2_Pricing'!B30)*'2_Pricing'!B6/'2_Pricing'!B19</ns0:f>
+        <ns0:v>0.7179216</ns0:v>
+      </ns0:c>
+      <ns0:c r="C86" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>fraction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D86" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>derived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E86" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Stricter than GM60 gate; point75% not same as confidence bound</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F86" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Rollout gate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="87" ht="48" customHeight="1" s="45">
+      <ns0:c r="A87" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pilot GM60 containment</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B87" s="56">
+        <ns0:f>B73*'1_Cost_Job'!B10/('2_Pricing'!B19*(1-'2_Pricing'!B32))</ns0:f>
+        <ns0:v>0.667712444444444</ns0:v>
+      </ns0:c>
+      <ns0:c r="C87" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>fraction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D87" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>derived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E87" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Volume-specific pilot healthy margin threshold</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F87" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pilot scenario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="88" ht="48" customHeight="1" s="45">
+      <ns0:c r="A88" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GM risk threshold</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B88" s="55" t="n">
+        <ns0:v>0.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="C88" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>fraction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D88" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>lab risk convention</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E88" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>For risk warning only; healthy GM target60%</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F88" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Lab Checkpoint3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="89" ht="48" customHeight="1" s="45">
+      <ns0:c r="A89" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Scorecard maximum</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B89" s="55" t="n">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="C89" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>points</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D89" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>lab convention</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E89" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Not a measured metric; score total maximum</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F89" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>3_Value_Metric!A10,A18</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="90" ht="48" customHeight="1" s="45">
+      <ns0:c r="A90" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Course track</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B90" s="55" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="C90" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>track</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D90" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>course identifier</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E90" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Track1 from uploaded template</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F90" s="54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>0_README!A2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
   </ns0:sheetData>
-  <ns0:autoFilter ref="A3:F78"/>
+  <ns0:autoFilter ref="A3:F90"/>
   <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ns0:pageSetup orientation="landscape" paperSize="8" fitToWidth="1"/>
 </ns0:worksheet>

</xml_diff>